<commit_message>
feat: optimize selective LKH, accelerate APGGS, add unit tests, and configure CI/CD for Render
</commit_message>
<xml_diff>
--- a/evaluation/results/apggs_ablation_results.xlsx
+++ b/evaluation/results/apggs_ablation_results.xlsx
@@ -488,7 +488,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>a280</t>
+          <t>kroa100</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -500,22 +500,22 @@
         <v>42</v>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>2579</v>
+        <v>21282</v>
       </c>
       <c r="G2" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
-        <v>17.85410141944885</v>
+        <v>0.6749694347381592</v>
       </c>
       <c r="I2" t="n">
-        <v>2579</v>
+        <v>21282</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -527,7 +527,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>a280</t>
+          <t>kroa100</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -539,34 +539,34 @@
         <v>42</v>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>2634</v>
+        <v>24000</v>
       </c>
       <c r="G3" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="H3" t="n">
-        <v>7.66502833366394</v>
+        <v>0.02741861343383789</v>
       </c>
       <c r="I3" t="n">
-        <v>2579</v>
+        <v>21282</v>
       </c>
       <c r="J3" t="n">
-        <v>55</v>
+        <v>2718</v>
       </c>
       <c r="K3" t="n">
-        <v>2.132609538580845</v>
+        <v>12.77135607555681</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>a280</t>
+          <t>kroa100</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -578,34 +578,34 @@
         <v>42</v>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>2625</v>
+        <v>21282</v>
       </c>
       <c r="G4" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="H4" t="n">
-        <v>5.06854248046875</v>
+        <v>0.6555314064025879</v>
       </c>
       <c r="I4" t="n">
-        <v>2579</v>
+        <v>21282</v>
       </c>
       <c r="J4" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1.783637068631252</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>a280</t>
+          <t>kroa100</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -617,34 +617,34 @@
         <v>42</v>
       </c>
       <c r="D5" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>2718</v>
+        <v>23267</v>
       </c>
       <c r="G5" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9378297328948975</v>
+        <v>0.03617119789123535</v>
       </c>
       <c r="I5" t="n">
-        <v>2579</v>
+        <v>21282</v>
       </c>
       <c r="J5" t="n">
-        <v>139</v>
+        <v>1985</v>
       </c>
       <c r="K5" t="n">
-        <v>5.389685924777045</v>
+        <v>9.327130908749178</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>a280</t>
+          <t>kroa100</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -656,28 +656,28 @@
         <v>42</v>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>2952</v>
+        <v>24249</v>
       </c>
       <c r="G6" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2403955459594727</v>
+        <v>0.01250672340393066</v>
       </c>
       <c r="I6" t="n">
-        <v>2579</v>
+        <v>21282</v>
       </c>
       <c r="J6" t="n">
-        <v>373</v>
+        <v>2967</v>
       </c>
       <c r="K6" t="n">
-        <v>14.46297014346646</v>
+        <v>13.94135889484071</v>
       </c>
     </row>
   </sheetData>

</xml_diff>